<commit_message>
P2: align sandbox runner + UC1 artifacts to the contract
run(ctx, **params), per-domain net scope, extension-preserving inputs,
write:outputs for live writes, non-blocking subprocess; UC1 workbooks
rebuilt to the reg/amt shape the UC1 pattern describes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/artifacts/uc1/week1.xlsx
+++ b/data/artifacts/uc1/week1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sales" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,99 +413,746 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Region</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>reg</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>amt</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1240.5</v>
+      <c r="D2" t="n">
+        <v>2022.13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>980</v>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>287.77</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>North</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Software</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2225.25</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1936.56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Services</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>870</v>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2177.35</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>South</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Software</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>1410.75</v>
+      <c r="D6" t="n">
+        <v>364.49</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1996.86</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1105.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1030.01</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1675.21</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1092.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1494.46</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1578.31</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>269.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1882.16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1814.94</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1830.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1691.07</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1882.2</v>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>590.72</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1329.65</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2253.32</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2326.94</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>194.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2212.67</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1645.29</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>454.51</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2177.32</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>746.42</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1543.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>326.91</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1457.74</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1071.23</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>870.54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>